<commit_message>
v2.5.0: thesis update from 98 new transcripts
- Cash conversion after stock pay (G7/H7/O7)
- Emerging uses EBIT basis for capital-heavy firms (E3/E12)
- Asset-Floor tangible-book route requires growing tangible book
- Red Flags: six new deterioration signals
- Criteria workbook and CLAUDE.md updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L62nuQP1Y9A1FWR9mxDHqX
</commit_message>
<xml_diff>
--- a/docs/criteria/Screener_Criteria.xlsx
+++ b/docs/criteria/Screener_Criteria.xlsx
@@ -209,10 +209,10 @@
     <t xml:space="preserve">Cash conversion</t>
   </si>
   <si>
-    <t xml:space="preserve">FCF / net income &gt;= 0.8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terry Smith states that profits must turn into cash, because his first test of a good company is a high return on capital in cash: cash delivered in a period divided by capital employed. A mentioned example: he put his own portfolio at about 25% on this measure (2022). Connor Haley states that free cash flow is a better guide than reported profits, because earnings and EBITDA "can be easily manipulated". No specific past example given.</t>
+    <t xml:space="preserve">(FCF - stock pay) / net income &gt;= 0.8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terry Smith states that profits must turn into cash, because his first test of a good company is a high return on capital in cash: cash delivered in a period divided by capital employed. A mentioned example: he put his own portfolio at about 25% on this measure (2022). Connor Haley states that free cash flow is a better guide than reported profits, because earnings and EBITDA "can be easily manipulated". No specific past example given. Jim Chanos states that stock pay is a real cost, because "It's compensation. You're diluting your shareholders by issuing them stock", yet it is routinely added back. No specific past example given; he said this of tech companies in general.</t>
   </si>
   <si>
     <t xml:space="preserve">Earnings quality.</t>
@@ -314,10 +314,10 @@
     <t xml:space="preserve">Already profitable</t>
   </si>
   <si>
-    <t xml:space="preserve">TTM and last-FY EBITDA &gt; 0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connor Haley states that already having positive EBITDA means the company is a proven business, not a cash burner, because most big winners were past the profit turning point and were not losing money and diluting shareholders to survive. A mentioned example: in Alta Fox's study of 104 multibaggers (2015-2020), 88% already had positive EBITDA five years earlier.</t>
+    <t xml:space="preserve">TTM and last-FY EBITDA &gt; 0 (EBIT &gt; 0 when D&amp;A &gt;= 50% of EBITDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connor Haley states that already having positive EBITDA means the company is a proven business, not a cash burner, because most big winners were past the profit turning point and were not losing money and diluting shareholders to survive. A mentioned example: in Alta Fox's study of 104 multibaggers (2015-2020), 88% already had positive EBITDA five years earlier. Tom Gayner states that EBITDA fits businesses with little capital spending but flatters capital-heavy ones, because when "the d number" is big, EBITDA stops describing what is really going on. A mentioned example: a radio station (EBITDA fair) versus a steel mill (EBITDA misleading). Nick Del Deo states that valuing a GPU cloud on EBITDA ignores "what it's costing you to create this thing". A mentioned example: CoreWeave, with very high EBITDA margins carried by depreciation (2025).</t>
   </si>
   <si>
     <t xml:space="preserve">Cuts cash-burning stories.</t>
@@ -467,10 +467,10 @@
     <t xml:space="preserve">Valuation</t>
   </si>
   <si>
-    <t xml:space="preserve">EV / EBITDA &lt;= 20x</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connor Haley states that a moderate EV/EBITDA means the thesis can work on profit growth alone, because "if your entire thesis rests on significant multiple expansion maybe it's not a great thesis". A mentioned example: in his study the median multibagger traded about 10x forward EBITDA five years earlier and re-rated to about 25x, with two-thirds of the return from multiple expansion. Chris Davis states that a reasonable starting multiple means your return is set by the business, because he assumes no re-rating: "We may get it, but it's nowhere in our models." A mentioned example: in 2026 his holdings at about 14x earnings offered a 7.5% earnings yield, versus about 3.8% for the market at 26x.</t>
+    <t xml:space="preserve">EV / EBITDA &lt;= 20x (EV / EBIT when D&amp;A &gt;= 50% of EBITDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connor Haley states that a moderate EV/EBITDA means the thesis can work on profit growth alone, because "if your entire thesis rests on significant multiple expansion maybe it's not a great thesis". A mentioned example: in his study the median multibagger traded about 10x forward EBITDA five years earlier and re-rated to about 25x, with two-thirds of the return from multiple expansion. Chris Davis states that a reasonable starting multiple means your return is set by the business, because he assumes no re-rating: "We may get it, but it's nowhere in our models." A mentioned example: in 2026 his holdings at about 14x earnings offered a 7.5% earnings yield, versus about 3.8% for the market at 26x. Tom Gayner states that EBITDA is "exactly inversely proportionate" in accuracy to how large depreciation is, because capital-heavy assets must be replaced. A mentioned example: radio station versus steel mill. So the screen values capital-heavy businesses on EV/EBIT.</t>
   </si>
   <si>
     <t xml:space="preserve">Return comes from growth, not multiple expansion.</t>
@@ -866,10 +866,10 @@
     <t xml:space="preserve">H7</t>
   </si>
   <si>
-    <t xml:space="preserve">FCF / net income &gt;= 0.7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Terry Smith states that turning profits into cash shows the returns are real, because he measures return on capital as cash delivered against the capital employed. A mentioned example: the MSCI World quality subset (high returns on capital, high margins, good cash conversion) beat the index in every rolling 10-year period since 1996. Connor Haley states that free cash flow is the number to trust, because earnings and EBITDA, unlike free cash flow, "can be easily manipulated". No specific past example given.</t>
+    <t xml:space="preserve">(FCF - stock pay) / net income &gt;= 0.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terry Smith states that turning profits into cash shows the returns are real, because he measures return on capital as cash delivered against the capital employed. A mentioned example: the MSCI World quality subset (high returns on capital, high margins, good cash conversion) beat the index in every rolling 10-year period since 1996. Connor Haley states that free cash flow is the number to trust, because earnings and EBITDA, unlike free cash flow, "can be easily manipulated". No specific past example given. Jim Chanos states that stock pay must be counted as a cost, because "It's compensation. You're diluting your shareholders", even though cash flow statements add it back. No specific past example given.</t>
   </si>
   <si>
     <t xml:space="preserve">H8</t>
@@ -1157,10 +1157,10 @@
     <t xml:space="preserve">O7</t>
   </si>
   <si>
-    <t xml:space="preserve">FCF / net income &gt;= 0.6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connor Haley states that relying on free cash flow means trusting the number hardest to fake, because earnings and EBITDA "can be easily manipulated". No specific past example given. Terry Smith states that good cash conversion is a mark of quality, because profits only count if they arrive as cash, so he measures return on capital in cash. A mentioned example: the MSCI World quality subset (high returns, high margins, good cash conversion) beat the index in every rolling 10-year period since 1996. Dan Sundheim states that profits that don't reconcile with the cash and unit economics can signal accounting abuse, because capitalizing costs that should be expensed lifts profit without bringing in cash. A mentioned example: Orthodontic Centers of America, where he found "the simplest form of accounting fraud".</t>
+    <t xml:space="preserve">(FCF - stock pay) / net income &gt;= 0.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connor Haley states that relying on free cash flow means trusting the number hardest to fake, because earnings and EBITDA "can be easily manipulated". No specific past example given. Terry Smith states that good cash conversion is a mark of quality, because profits only count if they arrive as cash, so he measures return on capital in cash. A mentioned example: the MSCI World quality subset (high returns, high margins, good cash conversion) beat the index in every rolling 10-year period since 1996. Dan Sundheim states that profits that don't reconcile with the cash and unit economics can signal accounting abuse, because capitalizing costs that should be expensed lifts profit without bringing in cash. A mentioned example: Orthodontic Centers of America, where he found "the simplest form of accounting fraud". Jim Chanos states that stock pay is a cost that cash flow hides, because "It's compensation. You're diluting your shareholders". No specific past example given.</t>
   </si>
   <si>
     <t xml:space="preserve">O8</t>
@@ -1328,10 +1328,10 @@
     <t xml:space="preserve">Below a hard floor</t>
   </si>
   <si>
-    <t xml:space="preserve">Market cap &lt;= 1.0x net cash, or price &lt;= 1.0x tangible book</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prem Watsa states that buying below cash per share gives you the rest of the business for free, because the cash alone covers the price, leaving plants and inventories as a bonus. A mentioned example: Fairfax bought Seagram at about $65 a share against roughly $70 of cash per share, and the stock doubled and tripled. Joel Greenblatt states that a stock selling at its cash, with a business not burning money, is a bargain worth a look, because management has no incentive to waste the cash and the business may turn into something: "almost like a free option". No specific past example given.</t>
+    <t xml:space="preserve">Market cap &lt;= 1.0x net cash, or price &lt;= 1.0x tangible book with tangible book per share not down over 3 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prem Watsa states that buying below cash per share gives you the rest of the business for free, because the cash alone covers the price, leaving plants and inventories as a bonus. A mentioned example: Fairfax bought Seagram at about $65 a share against roughly $70 of cash per share, and the stock doubled and tripled. Joel Greenblatt states that a stock selling at its cash, with a business not burning money, is a bargain worth a look, because management has no incentive to waste the cash and the business may turn into something: "almost like a free option". No specific past example given. Steve Eisman states that "buying a home builder below tangible book value ... when the builder is growing book value, usually works out", because a growing book shows the floor is real rather than eroding. A mentioned example: Meritage Homes below tangible book (2025).</t>
   </si>
   <si>
     <t xml:space="preserve">Hard downside floor (the thesis).</t>
@@ -1670,10 +1670,10 @@
     <t xml:space="preserve">Something is breaking</t>
   </si>
   <si>
-    <t xml:space="preserve">&gt;= 2 of: growth &lt; half its 3-yr rate; gross margin down 3 yrs; op margin down &gt;= 5 pts; TTM loss; dilution &gt;= 5%/yr; shrinking revenue</t>
-  </si>
-  <si>
-    <t xml:space="preserve">David Einhorn states that a short needs "over valuation combined with some kind of deterioration", because an expensive stock can stay expensive until the business visibly weakens. A mentioned example: in his bubble basket he would change his view on names once they "start showing real profits". Steve Cohen states that slowing growth on a high multiple is "a mix that doesn't give you much upside", because the price still assumes growth that is fading. No specific past example given; he said this of the market in May 2025.</t>
+    <t xml:space="preserve">&gt;= 2 of: growth &lt; half its 3-yr rate; gross margin down 3 yrs; op margin down &gt;= 5 pts; TTM loss; dilution &gt;= 5%/yr; shrinking revenue; profits above cash 2 yrs; negative operating cash flow; restructuring in &gt;= 4 of 5 yrs; acquisitions &gt; operating cash flow (3 yrs); inventory days at 5-yr high; heavy capex with negative FCF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">David Einhorn states that a short needs "over valuation combined with some kind of deterioration", because an expensive stock can stay expensive until the business visibly weakens. A mentioned example: in his bubble basket he would change his view on names once they "start showing real profits". Steve Cohen states that slowing growth on a high multiple is "a mix that doesn't give you much upside", because the price still assumes growth that is fading. No specific past example given; he said this of the market in May 2025. Jim Chanos states that "a lot of frauds have negative cash flow or have growing by acquisition", and that restructuring charges taken "10 out of the last 12 years" are not non-recurring. A mentioned example: IBM's recurring restructuring charges. Gavin Baker states that inventories at record highs warned of a downturn. A mentioned example: his February 2000 semiconductor sell call, when "days inventory were at all-time highs".</t>
   </si>
   <si>
     <t xml:space="preserve">Second half of the avoid case.</t>
@@ -2772,7 +2772,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
@@ -2971,7 +2971,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="2" t="s">
         <v>82</v>
       </c>
@@ -3228,7 +3228,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
         <v>82</v>
       </c>
@@ -4105,7 +4105,7 @@
         <v>277</v>
       </c>
     </row>
-    <row r="57" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="2" t="s">
         <v>252</v>
       </c>
@@ -4868,7 +4868,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="84" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="84" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="2" t="s">
         <v>354</v>
       </c>
@@ -5432,7 +5432,7 @@
       </c>
       <c r="I103" s="4"/>
     </row>
-    <row r="104" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="104" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="2" t="s">
         <v>420</v>
       </c>
@@ -6390,7 +6390,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="138" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="2" t="s">
         <v>533</v>
       </c>
@@ -7865,7 +7865,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="51" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
         <v>533</v>
       </c>

</xml_diff>

<commit_message>
v2.7.0: incremental SEC sync, slimmer workflows, ownership intel, Tech S-curve screen
- SEC daily-index sync + bulk zips; only filers re-downloaded; optional workbook
- Daily job exits on no new trading day; new background job for slow fills;
  publish skipped when data and site code are unchanged; cache pruning
- Twelve Data history once, extended from Massive; ECB FX; unpriceable memory;
  incremental splits; write-once descriptions for listed companies + peers
- Ownership card: 13F conviction, buyers/sellers vs previous quarter, insider
  open-market trades (Form 345) over 3 quarters
- Tech S-Curve Leaders screen (A1-A16) with thesis, criteria rows and tests
- Site text in qs/screen_text.py; Excel model in lazy site/model.js; fix direct
  company-page links rendering under the sidebar; CLAUDE.md trimmed (detail in docs/HANDOFF.md)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01L62nuQP1Y9A1FWR9mxDHqX
</commit_message>
<xml_diff>
--- a/docs/criteria/Screener_Criteria.xlsx
+++ b/docs/criteria/Screener_Criteria.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Summary" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Criteria!$A$1:$I$141</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Unverifiable!$A$1:$F$53</definedName>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Criteria!$A$1:$I$158</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">Unverifiable!$A$1:$F$59</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1656" uniqueCount="646">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1843" uniqueCount="717">
   <si>
     <t xml:space="preserve">Screen</t>
   </si>
@@ -1718,6 +1718,207 @@
     <t xml:space="preserve">Avg daily value traded &gt;= $1M</t>
   </si>
   <si>
+    <t xml:space="preserve">Tech S-Curve Leaders</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SIC 7370-7379 (software branch); 3570-3579, 3661-3679, 3825, 3827 (hardware branch); config allowlist</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ben Silver and David Tykocinski (Maverick) state that one screen should cover software and AI picks-and-shovels alike, because value in a technology wave moves between layers, "upstream" first and downstream later. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rules test economics, not the AI story.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Sacerdote states that an S-curve shows up as growth and rising margins together, because "when you get scurve and a rising margin your earnings don't grow linearly they grow exponentially"; seeing both needs several years of numbers. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Old numbers can hide a recent collapse; the screen needs the latest annual report. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Matches the Emerging screen's size floor: tiny filers have patchy data and are hard to own. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brad Gerstner states that growth means value in technology, because "the single greatest input to valuation technology is growth". No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Defining rule of the screen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">YTD (else latest FY) growth &gt;= 3-yr CAGR - 5 pts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Sacerdote states that a revenue miss means a broken tech stock, because "the biggest reason people blow up in Tech is they miss on revenue". Brad Gerstner adds that "every sell-side model on Wall Street has linear deceleration in growth rates", so a fade faster than that surprises the market. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catches the deceleration models assume away.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rule of 40 after stock pay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-yr revenue CAGR + 3-yr (FCF - SBC) / revenue &gt;= 40%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Philippe and Thomas Laffont (Coatue) state that growth plus profitability of 40 marks the strong cohort, because "growth in profitability yielding a rule of 40 was kind of the average of the cohort". Brad Gerstner and Bill Mylod state that stock pay is a real expense, so it is subtracted from free cash flow here. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth and cash generation in one test, net of stock pay.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software &gt;= 70%; hardware: gross margin up over 3 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Aaron Levie states that a low gross margin means a software company can never earn software margins, because at "40 50 60% gross margin, like there's just like no way you're going to have an operating margin [that] looks like a software company". Maverick states that hardware is different: the "sharpest revision torque" came "frequently against companies that had very low margin basis", so for hardware the test is a rising margin. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Room for software-like operating margins / pricing power.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Operating margin up over 3 yrs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alex Sacerdote states that rising margins on an S-curve mean exponential earnings, because "when you get scurve and a rising margin your earnings don't grow linearly they grow exponentially". No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Earnings compound faster than sales.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock pay vs free cash flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SBC &lt;= 20% of FCF (3 yrs); FCF &lt;= 0 fails</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capital allocation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brad Gerstner states that stock pay under a fifth of free cash flow marks a rare, disciplined company, because there are "maybe 10 names that are under 20% of their free cash flow as a percentage of stock-based compensation". Bill Mylod calls stock pay "the most single valuable expense". No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash flow belongs to shareholders, not staff.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share count growth &lt;= 1%/yr (3 yrs)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill Mylod states that a shrinking share count turns business growth into a bigger share-price gain, because "if the enterprise value has doubled, the share price has tripled" for a company that bought back stock. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Per-share value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Self-funded</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capex &lt;= 100% of operating cash flow (3 yrs) and net debt / EBITDA &lt;= 2.0x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Maverick states that today's AI build-out differs from the dot-com one because spending is "well under 100 percent" of operating cash flow. Gavin Baker asks whether spending is "funded out of debt or cash flows", and Bill Gurley warns that a "three to one ... debt to equity ratio" could be "a real painful ... downside". A mentioned example: the dot-com build-out versus today's cash-funded AI build-out.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Build-outs paid from own cash, not debt or new shares.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Return on new capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-yr incremental ROIC &gt;= 15% (capital-light growth counts as a pass)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Returns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill Gurley states that growth spending must be judged by "what's the return on the incremental investment". Michael Mauboussin states that growth creates value only when companies "earn above the opportunity cost of capital". No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth that creates value.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invested capital from balance-sheet tags; acquisitions distort.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Working capital</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Software: receivable days up &lt;= 10 over 3 yrs; hardware: inventory days not at a 5-yr high</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill Gurley states that slipping receivables mean a company is pulling revenue forward, because "their DSO's are just slipping out". Gavin Baker states that piling inventory signals a bust, because before the 2000 chip crash "customer inventories and days inventory were at all-time highs". A mentioned example: chip stocks in 2000.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early warning of channel stuffing or a demand air pocket.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market cap &gt;= $1B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Big enough to trade without moving the price. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Avg daily value traded &gt;= $5M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Must be able to build and exit a position. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A16</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV / sales &lt;= 3-yr growth in points / 3 (30% -&gt; 10x), max 15x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bill Gurley states that a high sales multiple needs high growth, because "if you want a 10x multiple you got be growing 30 35%". Leon Shaulov warns that winners "may not screen as the cheapest things in the world", so failing only this rule makes a 'wait for a better price' near miss. No specific past example given.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Price justified by growth; failing only this = 'wait for a better price'.</t>
+  </si>
+  <si>
     <t xml:space="preserve">'Cheap enough' rule (pass/fail)</t>
   </si>
   <si>
@@ -1784,6 +1985,12 @@
     <t xml:space="preserve">EV/sales &gt;= 6x (expensive = flag)</t>
   </si>
   <si>
+    <t xml:space="preserve">EV/sales &lt;= growth points / 3, max 15x</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Growth-adjusted multiple</t>
+  </si>
+  <si>
     <t xml:space="preserve">Answer: 9 of 13 screens have an absolute 'cheap enough' rule. None compares price to peers or to the company's own past multiples as a pass/fail rule.</t>
   </si>
   <si>
@@ -1899,6 +2106,12 @@
   </si>
   <si>
     <t xml:space="preserve">Short interest and insider-trade data not connected.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moat, S-curve stage (adoption share), depreciation policy for compute, AI disruption risk. Excluded by choice (Oct 2026): market position, net retention, AI share of sales, customer concentration, China/Taiwan exposure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not in XBRL financial data (dimensional or narrative).</t>
   </si>
   <si>
     <t xml:space="preserve">Kept (verifiable for most; gaps -&gt; Near misses with the reason)</t>
@@ -2523,7 +2736,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I158"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18"/>
@@ -6522,9 +6735,484 @@
       </c>
       <c r="I141" s="4"/>
     </row>
+    <row r="142" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A142" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B142" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C142" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D142" s="4" t="s">
+        <v>564</v>
+      </c>
+      <c r="E142" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="F142" s="4" t="s">
+        <v>565</v>
+      </c>
+      <c r="G142" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="H142" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I142" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="143" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A143" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B143" s="3" t="s">
+        <v>567</v>
+      </c>
+      <c r="C143" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D143" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E143" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F143" s="4" t="s">
+        <v>568</v>
+      </c>
+      <c r="G143" s="4" t="s">
+        <v>259</v>
+      </c>
+      <c r="H143" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I143" s="4"/>
+    </row>
+    <row r="144" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A144" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B144" s="3" t="s">
+        <v>569</v>
+      </c>
+      <c r="C144" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D144" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="E144" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F144" s="4" t="s">
+        <v>570</v>
+      </c>
+      <c r="G144" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H144" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I144" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="145" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A145" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>571</v>
+      </c>
+      <c r="C145" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D145" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="E145" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="F145" s="4" t="s">
+        <v>572</v>
+      </c>
+      <c r="G145" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="H145" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I145" s="4"/>
+    </row>
+    <row r="146" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>573</v>
+      </c>
+      <c r="C146" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D146" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E146" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F146" s="4" t="s">
+        <v>574</v>
+      </c>
+      <c r="G146" s="4" t="s">
+        <v>575</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I146" s="4"/>
+    </row>
+    <row r="147" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B147" s="3" t="s">
+        <v>576</v>
+      </c>
+      <c r="C147" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D147" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="E147" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="F147" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="G147" s="4" t="s">
+        <v>579</v>
+      </c>
+      <c r="H147" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I147" s="4"/>
+    </row>
+    <row r="148" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B148" s="3" t="s">
+        <v>580</v>
+      </c>
+      <c r="C148" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="D148" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="E148" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F148" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="G148" s="4" t="s">
+        <v>584</v>
+      </c>
+      <c r="H148" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I148" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="149" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B149" s="3" t="s">
+        <v>585</v>
+      </c>
+      <c r="C149" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D149" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="E149" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F149" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="G149" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="H149" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I149" s="4"/>
+    </row>
+    <row r="150" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A150" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B150" s="3" t="s">
+        <v>589</v>
+      </c>
+      <c r="C150" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D150" s="4" t="s">
+        <v>590</v>
+      </c>
+      <c r="E150" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F150" s="4" t="s">
+        <v>591</v>
+      </c>
+      <c r="G150" s="4" t="s">
+        <v>592</v>
+      </c>
+      <c r="H150" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I150" s="4"/>
+    </row>
+    <row r="151" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A151" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B151" s="3" t="s">
+        <v>593</v>
+      </c>
+      <c r="C151" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="D151" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="E151" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="F151" s="4" t="s">
+        <v>597</v>
+      </c>
+      <c r="G151" s="4" t="s">
+        <v>598</v>
+      </c>
+      <c r="H151" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I151" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="152" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A152" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B152" s="3" t="s">
+        <v>599</v>
+      </c>
+      <c r="C152" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D152" s="4" t="s">
+        <v>600</v>
+      </c>
+      <c r="E152" s="3" t="s">
+        <v>596</v>
+      </c>
+      <c r="F152" s="4" t="s">
+        <v>601</v>
+      </c>
+      <c r="G152" s="4" t="s">
+        <v>602</v>
+      </c>
+      <c r="H152" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I152" s="4"/>
+    </row>
+    <row r="153" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A153" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B153" s="3" t="s">
+        <v>603</v>
+      </c>
+      <c r="C153" s="2" t="s">
+        <v>604</v>
+      </c>
+      <c r="D153" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="E153" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="F153" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="G153" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="H153" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I153" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="154" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A154" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B154" s="3" t="s">
+        <v>608</v>
+      </c>
+      <c r="C154" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="D154" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="E154" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="F154" s="4" t="s">
+        <v>612</v>
+      </c>
+      <c r="G154" s="4" t="s">
+        <v>613</v>
+      </c>
+      <c r="H154" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I154" s="4" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="155" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A155" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B155" s="3" t="s">
+        <v>615</v>
+      </c>
+      <c r="C155" s="2" t="s">
+        <v>616</v>
+      </c>
+      <c r="D155" s="4" t="s">
+        <v>617</v>
+      </c>
+      <c r="E155" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>618</v>
+      </c>
+      <c r="G155" s="4" t="s">
+        <v>619</v>
+      </c>
+      <c r="H155" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I155" s="4"/>
+    </row>
+    <row r="156" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A156" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B156" s="3" t="s">
+        <v>620</v>
+      </c>
+      <c r="C156" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="D156" s="4" t="s">
+        <v>621</v>
+      </c>
+      <c r="E156" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>622</v>
+      </c>
+      <c r="G156" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H156" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I156" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="157" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A157" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B157" s="3" t="s">
+        <v>623</v>
+      </c>
+      <c r="C157" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D157" s="4" t="s">
+        <v>624</v>
+      </c>
+      <c r="E157" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="F157" s="4" t="s">
+        <v>625</v>
+      </c>
+      <c r="G157" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="H157" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="I157" s="4"/>
+    </row>
+    <row r="158" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A158" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B158" s="3" t="s">
+        <v>626</v>
+      </c>
+      <c r="C158" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="D158" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="E158" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="F158" s="4" t="s">
+        <v>628</v>
+      </c>
+      <c r="G158" s="4" t="s">
+        <v>629</v>
+      </c>
+      <c r="H158" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="I158" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I141"/>
-  <conditionalFormatting sqref="H2:H141">
+  <autoFilter ref="A1:I158"/>
+  <conditionalFormatting sqref="H2:H158">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
       <formula>$H2="Easy"</formula>
     </cfRule>
@@ -6538,7 +7226,7 @@
       <formula>$H2="n/a"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A2:I141">
+  <conditionalFormatting sqref="A2:I158">
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10">
       <formula>$E2="Valuation"</formula>
     </cfRule>
@@ -6559,7 +7247,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -6575,19 +7263,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>563</v>
+        <v>630</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>564</v>
+        <v>631</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>565</v>
+        <v>632</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>566</v>
+        <v>633</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>567</v>
+        <v>634</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6595,19 +7283,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>568</v>
+        <v>635</v>
       </c>
       <c r="C2" s="4" t="s">
         <v>249</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6615,19 +7303,19 @@
         <v>82</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>572</v>
+        <v>639</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6635,19 +7323,19 @@
         <v>154</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>574</v>
+        <v>641</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6655,19 +7343,19 @@
         <v>186</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>575</v>
+        <v>642</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>249</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6675,19 +7363,19 @@
         <v>252</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>575</v>
+        <v>642</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>249</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6695,19 +7383,19 @@
         <v>290</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>576</v>
+        <v>643</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>577</v>
+        <v>644</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6718,16 +7406,16 @@
         <v>356</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>578</v>
+        <v>645</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6735,19 +7423,19 @@
         <v>359</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>579</v>
+        <v>646</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6755,19 +7443,19 @@
         <v>395</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>580</v>
+        <v>647</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6775,19 +7463,19 @@
         <v>426</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>581</v>
+        <v>648</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>577</v>
+        <v>644</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6795,19 +7483,19 @@
         <v>457</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>582</v>
+        <v>649</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>583</v>
+        <v>650</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6815,19 +7503,19 @@
         <v>503</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>574</v>
+        <v>641</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6835,44 +7523,54 @@
         <v>539</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>584</v>
+        <v>651</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>573</v>
+        <v>640</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>569</v>
+        <v>636</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>570</v>
+        <v>637</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>571</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="s">
-        <v>585</v>
-      </c>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
-      <c r="F16" s="5"/>
+        <v>638</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>652</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>653</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>636</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>637</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>638</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="s">
-        <v>586</v>
-      </c>
-      <c r="B17" s="6"/>
-      <c r="C17" s="6"/>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="6"/>
+      <c r="A17" s="5" t="s">
+        <v>654</v>
+      </c>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>587</v>
+        <v>655</v>
       </c>
       <c r="B18" s="6"/>
       <c r="C18" s="6"/>
@@ -6880,11 +7578,21 @@
       <c r="E18" s="6"/>
       <c r="F18" s="6"/>
     </row>
+    <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="s">
+        <v>656</v>
+      </c>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+    </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A16:F16"/>
     <mergeCell ref="A17:F17"/>
     <mergeCell ref="A18:F18"/>
+    <mergeCell ref="A19:F19"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -6901,7 +7609,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -6920,16 +7628,16 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>588</v>
+        <v>657</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>589</v>
+        <v>658</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>590</v>
+        <v>659</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>591</v>
+        <v>660</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6937,19 +7645,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>592</v>
+        <v>661</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>593</v>
+        <v>662</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>595</v>
+        <v>664</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>596</v>
+        <v>665</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6957,19 +7665,19 @@
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>597</v>
+        <v>666</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>598</v>
+        <v>667</v>
       </c>
       <c r="D3" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6977,19 +7685,19 @@
         <v>82</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>602</v>
+        <v>671</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6997,19 +7705,19 @@
         <v>154</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>603</v>
+        <v>672</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>604</v>
+        <v>673</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7017,19 +7725,19 @@
         <v>186</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>605</v>
+        <v>674</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>606</v>
+        <v>675</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>595</v>
+        <v>664</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>607</v>
+        <v>676</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7037,19 +7745,19 @@
         <v>186</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>608</v>
+        <v>677</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7057,19 +7765,19 @@
         <v>252</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>605</v>
+        <v>674</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>606</v>
+        <v>675</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>595</v>
+        <v>664</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>607</v>
+        <v>676</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7077,19 +7785,19 @@
         <v>252</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>609</v>
+        <v>678</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>610</v>
+        <v>679</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7097,19 +7805,19 @@
         <v>290</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>611</v>
+        <v>680</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>612</v>
+        <v>681</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7117,19 +7825,19 @@
         <v>325</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>613</v>
+        <v>682</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>614</v>
+        <v>683</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7137,19 +7845,19 @@
         <v>359</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>605</v>
+        <v>674</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>606</v>
+        <v>675</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>595</v>
+        <v>664</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>607</v>
+        <v>676</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7157,19 +7865,19 @@
         <v>359</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>615</v>
+        <v>684</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>616</v>
+        <v>685</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7177,19 +7885,19 @@
         <v>395</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>617</v>
+        <v>686</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7197,19 +7905,19 @@
         <v>426</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>618</v>
+        <v>687</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7217,19 +7925,19 @@
         <v>457</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>619</v>
+        <v>688</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>599</v>
+        <v>668</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7237,19 +7945,19 @@
         <v>503</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>620</v>
+        <v>689</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>621</v>
+        <v>690</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>600</v>
+        <v>669</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7257,59 +7965,59 @@
         <v>539</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>601</v>
+        <v>670</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>622</v>
+        <v>691</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>594</v>
+        <v>663</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>623</v>
+        <v>692</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>600</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>670</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>693</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>663</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>694</v>
+      </c>
+      <c r="F19" s="4" t="s">
+        <v>669</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B20" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="4" t="s">
+      <c r="C20" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="D19" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E19" s="4" t="s">
+      <c r="D20" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E20" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="F19" s="4" t="s">
-        <v>625</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C20" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="D20" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E20" s="4" t="s">
-        <v>109</v>
-      </c>
       <c r="F20" s="4" t="s">
-        <v>626</v>
+        <v>696</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7317,39 +8025,39 @@
         <v>82</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>122</v>
+        <v>105</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>123</v>
+        <v>106</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>126</v>
+        <v>109</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>627</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
         <v>82</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>133</v>
+        <v>122</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>134</v>
+        <v>123</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>628</v>
+        <v>698</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7357,19 +8065,19 @@
         <v>82</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E23" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7377,39 +8085,39 @@
         <v>82</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E24" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="2" t="s">
-        <v>154</v>
+        <v>82</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>627</v>
+        <v>699</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7417,19 +8125,19 @@
         <v>154</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>24</v>
+        <v>155</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>25</v>
+        <v>156</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>627</v>
+        <v>698</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7437,79 +8145,79 @@
         <v>154</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>165</v>
+        <v>24</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>166</v>
+        <v>25</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
         <v>154</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="2" t="s">
         <v>154</v>
       </c>
       <c r="B29" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C29" s="4" t="s">
+      <c r="C30" s="4" t="s">
         <v>181</v>
       </c>
-      <c r="D29" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E29" s="4" t="s">
+      <c r="D30" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E30" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F29" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="2" t="s">
-        <v>186</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="D30" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E30" s="4" t="s">
-        <v>206</v>
-      </c>
       <c r="F30" s="4" t="s">
-        <v>625</v>
+        <v>699</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7517,39 +8225,39 @@
         <v>186</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="F31" s="4" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="B32" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C32" s="4" t="s">
         <v>232</v>
       </c>
-      <c r="D31" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E31" s="4" t="s">
+      <c r="D32" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E32" s="4" t="s">
         <v>235</v>
       </c>
-      <c r="F31" s="4" t="s">
-        <v>630</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="2" t="s">
-        <v>290</v>
-      </c>
-      <c r="B32" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C32" s="4" t="s">
-        <v>311</v>
-      </c>
-      <c r="D32" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>138</v>
-      </c>
       <c r="F32" s="4" t="s">
-        <v>628</v>
+        <v>701</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7557,19 +8265,19 @@
         <v>290</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>316</v>
+        <v>133</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>317</v>
+        <v>311</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E33" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7577,79 +8285,79 @@
         <v>290</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>321</v>
+        <v>316</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>322</v>
+        <v>317</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E34" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="2" t="s">
-        <v>325</v>
+        <v>290</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>355</v>
+        <v>321</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>356</v>
+        <v>322</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E35" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="2" t="s">
-        <v>359</v>
+        <v>325</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>369</v>
+        <v>355</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>370</v>
+        <v>356</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>373</v>
+        <v>138</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>631</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="2" t="s">
         <v>359</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>133</v>
+        <v>369</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>181</v>
+        <v>370</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>138</v>
+        <v>373</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>628</v>
+        <v>702</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7657,39 +8365,39 @@
         <v>359</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>392</v>
+        <v>181</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E38" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>395</v>
+        <v>359</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>133</v>
+        <v>145</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>181</v>
+        <v>392</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E39" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7697,79 +8405,79 @@
         <v>395</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>145</v>
+        <v>133</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>423</v>
+        <v>181</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E40" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="2" t="s">
-        <v>426</v>
+        <v>395</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>438</v>
+        <v>145</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>439</v>
+        <v>423</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>442</v>
+        <v>138</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="2" t="s">
         <v>426</v>
       </c>
       <c r="B42" s="2" t="s">
+        <v>438</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>439</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="B43" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C42" s="4" t="s">
+      <c r="C43" s="4" t="s">
         <v>311</v>
       </c>
-      <c r="D42" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E42" s="4" t="s">
+      <c r="D43" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E43" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F42" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2" t="s">
-        <v>457</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>472</v>
-      </c>
-      <c r="C43" s="4" t="s">
-        <v>473</v>
-      </c>
-      <c r="D43" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E43" s="4" t="s">
-        <v>476</v>
-      </c>
       <c r="F43" s="4" t="s">
-        <v>632</v>
+        <v>699</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7777,39 +8485,39 @@
         <v>457</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>478</v>
+        <v>472</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>479</v>
+        <v>473</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E44" s="4" t="s">
-        <v>482</v>
+        <v>476</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>632</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
         <v>457</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>486</v>
+        <v>478</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>487</v>
+        <v>479</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E45" s="4" t="s">
-        <v>490</v>
+        <v>482</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>628</v>
+        <v>703</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7817,79 +8525,79 @@
         <v>457</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>133</v>
+        <v>486</v>
       </c>
       <c r="C46" s="4" t="s">
-        <v>492</v>
+        <v>487</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>138</v>
+        <v>490</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="2" t="s">
         <v>457</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>497</v>
+        <v>133</v>
       </c>
       <c r="C47" s="4" t="s">
-        <v>498</v>
+        <v>492</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>502</v>
+        <v>138</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>627</v>
+        <v>699</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="2" t="s">
-        <v>503</v>
+        <v>457</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>511</v>
+        <v>497</v>
       </c>
       <c r="C48" s="4" t="s">
-        <v>512</v>
+        <v>498</v>
       </c>
       <c r="D48" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>515</v>
+        <v>502</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>633</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="2" t="s">
         <v>503</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>175</v>
+        <v>511</v>
       </c>
       <c r="C49" s="4" t="s">
-        <v>176</v>
+        <v>512</v>
       </c>
       <c r="D49" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>138</v>
+        <v>515</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>628</v>
+        <v>704</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7897,83 +8605,203 @@
         <v>503</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>133</v>
+        <v>175</v>
       </c>
       <c r="C50" s="4" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="D50" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E50" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>628</v>
+        <v>699</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="2" t="s">
-        <v>539</v>
+        <v>503</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>547</v>
+        <v>133</v>
       </c>
       <c r="C51" s="4" t="s">
-        <v>548</v>
+        <v>181</v>
       </c>
       <c r="D51" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E51" s="4" t="s">
         <v>138</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>628</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="2" t="s">
         <v>539</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>552</v>
+        <v>547</v>
       </c>
       <c r="C52" s="4" t="s">
-        <v>553</v>
+        <v>548</v>
       </c>
       <c r="D52" s="4" t="s">
-        <v>624</v>
+        <v>695</v>
       </c>
       <c r="E52" s="4" t="s">
-        <v>556</v>
+        <v>138</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>629</v>
-      </c>
-    </row>
-    <row r="53" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="2" t="s">
         <v>539</v>
       </c>
       <c r="B53" s="2" t="s">
+        <v>552</v>
+      </c>
+      <c r="C53" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="D53" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E53" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="F53" s="4" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2" t="s">
+        <v>539</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C53" s="4" t="s">
+      <c r="C54" s="4" t="s">
         <v>558</v>
       </c>
-      <c r="D53" s="4" t="s">
-        <v>624</v>
-      </c>
-      <c r="E53" s="4" t="s">
+      <c r="D54" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E54" s="4" t="s">
         <v>138</v>
       </c>
-      <c r="F53" s="4" t="s">
-        <v>628</v>
+      <c r="F54" s="4" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>581</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F55" s="4" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>594</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>595</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="F56" s="4" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>609</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>614</v>
+      </c>
+      <c r="F57" s="4" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="C58" s="4" t="s">
+        <v>621</v>
+      </c>
+      <c r="D58" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F58" s="4" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>563</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>627</v>
+      </c>
+      <c r="D59" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="E59" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>699</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F53"/>
+  <autoFilter ref="A1:F59"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -7990,7 +8818,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -8009,16 +8837,16 @@
         <v>75</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>571</v>
+        <v>638</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>250</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>634</v>
+        <v>705</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>635</v>
+        <v>706</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8026,19 +8854,19 @@
         <v>9</v>
       </c>
       <c r="B2" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A2,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A2,Criteria!$H$2:$H$158,"Easy")</f>
         <v>11</v>
       </c>
       <c r="C2" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A2,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A2,Criteria!$H$2:$H$158,"Partly")</f>
         <v>1</v>
       </c>
       <c r="D2" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A2,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A2,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E2" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A2,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A2,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F2" s="8" t="n">
@@ -8055,19 +8883,19 @@
         <v>82</v>
       </c>
       <c r="B3" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A3,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A3,Criteria!$H$2:$H$158,"Easy")</f>
         <v>9</v>
       </c>
       <c r="C3" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A3,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A3,Criteria!$H$2:$H$158,"Partly")</f>
         <v>5</v>
       </c>
       <c r="D3" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A3,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A3,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E3" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A3,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A3,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F3" s="8" t="n">
@@ -8084,19 +8912,19 @@
         <v>154</v>
       </c>
       <c r="B4" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A4,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A4,Criteria!$H$2:$H$158,"Easy")</f>
         <v>2</v>
       </c>
       <c r="C4" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A4,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A4,Criteria!$H$2:$H$158,"Partly")</f>
         <v>5</v>
       </c>
       <c r="D4" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A4,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A4,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E4" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A4,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A4,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F4" s="8" t="n">
@@ -8113,19 +8941,19 @@
         <v>186</v>
       </c>
       <c r="B5" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A5,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A5,Criteria!$H$2:$H$158,"Easy")</f>
         <v>12</v>
       </c>
       <c r="C5" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A5,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A5,Criteria!$H$2:$H$158,"Partly")</f>
         <v>2</v>
       </c>
       <c r="D5" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A5,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A5,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E5" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A5,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A5,Criteria!$H$2:$H$158,"n/a")</f>
         <v>1</v>
       </c>
       <c r="F5" s="8" t="n">
@@ -8142,19 +8970,19 @@
         <v>252</v>
       </c>
       <c r="B6" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A6,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A6,Criteria!$H$2:$H$158,"Easy")</f>
         <v>10</v>
       </c>
       <c r="C6" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A6,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A6,Criteria!$H$2:$H$158,"Partly")</f>
         <v>0</v>
       </c>
       <c r="D6" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A6,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A6,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E6" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A6,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A6,Criteria!$H$2:$H$158,"n/a")</f>
         <v>1</v>
       </c>
       <c r="F6" s="8" t="n">
@@ -8171,19 +8999,19 @@
         <v>290</v>
       </c>
       <c r="B7" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A7,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A7,Criteria!$H$2:$H$158,"Easy")</f>
         <v>5</v>
       </c>
       <c r="C7" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A7,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A7,Criteria!$H$2:$H$158,"Partly")</f>
         <v>3</v>
       </c>
       <c r="D7" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A7,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A7,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E7" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A7,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A7,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F7" s="8" t="n">
@@ -8200,19 +9028,19 @@
         <v>325</v>
       </c>
       <c r="B8" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A8,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A8,Criteria!$H$2:$H$158,"Easy")</f>
         <v>8</v>
       </c>
       <c r="C8" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A8,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A8,Criteria!$H$2:$H$158,"Partly")</f>
         <v>1</v>
       </c>
       <c r="D8" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A8,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A8,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E8" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A8,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A8,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F8" s="8" t="n">
@@ -8229,19 +9057,19 @@
         <v>359</v>
       </c>
       <c r="B9" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A9,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A9,Criteria!$H$2:$H$158,"Easy")</f>
         <v>9</v>
       </c>
       <c r="C9" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A9,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A9,Criteria!$H$2:$H$158,"Partly")</f>
         <v>3</v>
       </c>
       <c r="D9" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A9,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A9,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E9" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A9,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A9,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F9" s="8" t="n">
@@ -8258,19 +9086,19 @@
         <v>395</v>
       </c>
       <c r="B10" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A10,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A10,Criteria!$H$2:$H$158,"Easy")</f>
         <v>9</v>
       </c>
       <c r="C10" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A10,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A10,Criteria!$H$2:$H$158,"Partly")</f>
         <v>2</v>
       </c>
       <c r="D10" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A10,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A10,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E10" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A10,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A10,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F10" s="8" t="n">
@@ -8287,19 +9115,19 @@
         <v>426</v>
       </c>
       <c r="B11" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A11,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A11,Criteria!$H$2:$H$158,"Easy")</f>
         <v>8</v>
       </c>
       <c r="C11" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A11,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A11,Criteria!$H$2:$H$158,"Partly")</f>
         <v>2</v>
       </c>
       <c r="D11" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A11,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A11,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E11" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A11,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A11,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F11" s="8" t="n">
@@ -8316,19 +9144,19 @@
         <v>457</v>
       </c>
       <c r="B12" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A12,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A12,Criteria!$H$2:$H$158,"Easy")</f>
         <v>7</v>
       </c>
       <c r="C12" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A12,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A12,Criteria!$H$2:$H$158,"Partly")</f>
         <v>5</v>
       </c>
       <c r="D12" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A12,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A12,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E12" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A12,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A12,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F12" s="8" t="n">
@@ -8345,19 +9173,19 @@
         <v>503</v>
       </c>
       <c r="B13" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A13,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A13,Criteria!$H$2:$H$158,"Easy")</f>
         <v>9</v>
       </c>
       <c r="C13" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A13,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A13,Criteria!$H$2:$H$158,"Partly")</f>
         <v>3</v>
       </c>
       <c r="D13" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A13,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A13,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E13" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A13,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A13,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F13" s="8" t="n">
@@ -8374,19 +9202,19 @@
         <v>539</v>
       </c>
       <c r="B14" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A14,Criteria!$H$2:$H$141,"Easy")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A14,Criteria!$H$2:$H$158,"Easy")</f>
         <v>4</v>
       </c>
       <c r="C14" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A14,Criteria!$H$2:$H$141,"Partly")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A14,Criteria!$H$2:$H$158,"Partly")</f>
         <v>3</v>
       </c>
       <c r="D14" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A14,Criteria!$H$2:$H$141,"No")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A14,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
       <c r="E14" s="8" t="n">
-        <f aca="false">COUNTIFS(Criteria!$A$2:$A$141,$A14,Criteria!$H$2:$H$141,"n/a")</f>
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A14,Criteria!$H$2:$H$158,"n/a")</f>
         <v>0</v>
       </c>
       <c r="F14" s="8" t="n">
@@ -8400,57 +9228,73 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>636</v>
-      </c>
-      <c r="B15" s="10" t="n">
-        <f aca="false">SUM(B2:B14)</f>
-        <v>103</v>
-      </c>
-      <c r="C15" s="10" t="n">
-        <f aca="false">SUM(C2:C14)</f>
-        <v>35</v>
-      </c>
-      <c r="D15" s="10" t="n">
-        <f aca="false">SUM(D2:D14)</f>
+        <v>563</v>
+      </c>
+      <c r="B15" s="8" t="n">
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A15,Criteria!$H$2:$H$158,"Easy")</f>
+        <v>12</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A15,Criteria!$H$2:$H$158,"Partly")</f>
+        <v>5</v>
+      </c>
+      <c r="D15" s="8" t="n">
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A15,Criteria!$H$2:$H$158,"No")</f>
         <v>0</v>
       </c>
-      <c r="E15" s="10" t="n">
-        <f aca="false">SUM(E2:E14)</f>
+      <c r="E15" s="8" t="n">
+        <f aca="false">COUNTIFS(Criteria!$A$2:$A$158,$A15,Criteria!$H$2:$H$158,"n/a")</f>
+        <v>0</v>
+      </c>
+      <c r="F15" s="8" t="n">
+        <f aca="false">SUM(B15:E15)</f>
+        <v>17</v>
+      </c>
+      <c r="G15" s="9" t="n">
+        <f aca="false">IF(F15=0,0,B15/F15)</f>
+        <v>0.705882352941177</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>707</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <f aca="false">SUM(B2:B15)</f>
+        <v>115</v>
+      </c>
+      <c r="C16" s="10" t="n">
+        <f aca="false">SUM(C2:C15)</f>
+        <v>40</v>
+      </c>
+      <c r="D16" s="10" t="n">
+        <f aca="false">SUM(D2:D15)</f>
+        <v>0</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <f aca="false">SUM(E2:E15)</f>
         <v>2</v>
       </c>
-      <c r="F15" s="10" t="n">
-        <f aca="false">SUM(F2:F14)</f>
-        <v>140</v>
-      </c>
-      <c r="G15" s="11" t="n">
-        <f aca="false">IF(F15=0,0,B15/F15)</f>
-        <v>0.735714285714286</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>637</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>638</v>
-      </c>
-      <c r="C18" s="6"/>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="G18" s="6"/>
+      <c r="F16" s="10" t="n">
+        <f aca="false">SUM(F2:F15)</f>
+        <v>157</v>
+      </c>
+      <c r="G16" s="11" t="n">
+        <f aca="false">IF(F16=0,0,B16/F16)</f>
+        <v>0.732484076433121</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>708</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>75</v>
+      <c r="A19" s="13" t="s">
+        <v>15</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>639</v>
+        <v>709</v>
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
@@ -8459,11 +9303,11 @@
       <c r="G19" s="6"/>
     </row>
     <row r="20" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="15" t="s">
-        <v>571</v>
+      <c r="A20" s="14" t="s">
+        <v>75</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>640</v>
+        <v>710</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
@@ -8472,11 +9316,11 @@
       <c r="G20" s="6"/>
     </row>
     <row r="21" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="16" t="s">
-        <v>250</v>
+      <c r="A21" s="15" t="s">
+        <v>638</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>641</v>
+        <v>711</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
@@ -8485,11 +9329,11 @@
       <c r="G21" s="6"/>
     </row>
     <row r="22" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="12" t="s">
-        <v>642</v>
+      <c r="A22" s="16" t="s">
+        <v>250</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>643</v>
+        <v>712</v>
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
@@ -8499,10 +9343,10 @@
     </row>
     <row r="23" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="12" t="s">
-        <v>644</v>
+        <v>713</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>645</v>
+        <v>714</v>
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
@@ -8510,14 +9354,27 @@
       <c r="F23" s="6"/>
       <c r="G23" s="6"/>
     </row>
+    <row r="24" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="12" t="s">
+        <v>715</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>716</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+    </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B19:G19"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B21:G21"/>
     <mergeCell ref="B22:G22"/>
     <mergeCell ref="B23:G23"/>
+    <mergeCell ref="B24:G24"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>